<commit_message>
Finished unit testing savings account everything functions as intended
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_savings_account.xlsx
+++ b/tests/A02_pixell_test_plan_savings_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Updated Assignments ISD\assignment_02\given_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E5394E5-D09B-4C82-AD73-79542EE783C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{9E5394E5-D09B-4C82-AD73-79542EE783C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D5DAD34-46F4-4454-A8CC-943CDADFDE8F}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="25185" windowHeight="13845" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-105" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -233,9 +233,6 @@
     <t>balance less than minimum balance</t>
   </si>
   <si>
-    <t>Student Name</t>
-  </si>
-  <si>
     <t>Attributes are set to parameter values.</t>
   </si>
   <si>
@@ -246,6 +243,45 @@
   </si>
   <si>
     <t>balance  equal to minimum balance</t>
+  </si>
+  <si>
+    <t>Trevor Donald</t>
+  </si>
+  <si>
+    <t>SavingsAccount(123, 404, 1050.50, datetime.date(2025, 9, 29), 150.00)</t>
+  </si>
+  <si>
+    <t>SavingsAccount(123, 404, 150, datetime.date(2025, 9, 29), 150.00)</t>
+  </si>
+  <si>
+    <t>SavingsAccount(123, 404, 100, datetime.date(2025, 9, 29), 150.00)</t>
+  </si>
+  <si>
+    <t>SavingsAccount(123, 404, 1050.50, datetime.date(2025, 9, 29), "150.00")</t>
+  </si>
+  <si>
+    <t>account_number = 123 client_number = 404        balance = 1050.50  date_created = datetime.date(2025, 9, 29)       minum_balance = 150</t>
+  </si>
+  <si>
+    <t>minimum_balance = "150.00"</t>
+  </si>
+  <si>
+    <t>minimum_balance = 50.00</t>
+  </si>
+  <si>
+    <t>SavingsAccount.get_service_charges()</t>
+  </si>
+  <si>
+    <t>print(SavingsAccount)</t>
+  </si>
+  <si>
+    <t>service_charge = 0.50</t>
+  </si>
+  <si>
+    <t>service_charge = 1</t>
+  </si>
+  <si>
+    <t>Account Number: 123 Balance: $1,050.50  Minimum Balance: $150.00 Account Type: Savings</t>
   </si>
 </sst>
 </file>
@@ -1179,7 +1215,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="18"/>
     </row>
@@ -1223,11 +1259,17 @@
         <v>8</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+        <v>16</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
@@ -1239,9 +1281,15 @@
       <c r="D8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
+      <c r="E8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
@@ -1251,11 +1299,17 @@
         <v>13</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+        <v>18</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
@@ -1265,11 +1319,17 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+        <v>19</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
@@ -1281,9 +1341,15 @@
       <c r="D11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11">
@@ -1293,11 +1359,17 @@
         <v>11</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="11">

</xml_diff>